<commit_message>
README con indice, seguridad, Docker, CI/CD, diagramas y evidencias
</commit_message>
<xml_diff>
--- a/docs/roles-blue-velvet.xlsx
+++ b/docs/roles-blue-velvet.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roles" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matriz de permisos" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Roles" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Matriz de permisos" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -620,7 +620,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -1271,6 +1271,134 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Iniciar sesion y obtener token JWT</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>POST /api/v1/auth/login</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Registrarse como cliente</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>POST /api/v1/auth/registro</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Consultar el usuario autenticado</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>GET /api/v1/auth/me</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Consultar historial de eventos (MongoDB)</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>GET /api/v1/eventos</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Despliegue del frontend, documentos de arquitectura y evidencias
</commit_message>
<xml_diff>
--- a/docs/roles-blue-velvet.xlsx
+++ b/docs/roles-blue-velvet.xlsx
@@ -512,14 +512,17 @@
 - Crear modificadores
 - Ver la carta y el detalle de cada coctel
 - Consultar todas las comandas y filtrarlas por estado
-- Cancelar comandas en estado RECIBIDO</t>
+- Cancelar comandas en estado RECIBIDO
+- Crear, editar, eliminar y marcar como agotados los platos de la cocina
+- Consultar la agenda de reservas y marcarlas como cumplidas o canceladas</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
           <t>- Crear comandas
 - Cambiar el licor de un coctel de una comanda
-- Avanzar el estado de una comanda en el tablero del bartender</t>
+- Avanzar el estado de una comanda en el tablero del bartender
+- Calificar productos</t>
         </is>
       </c>
     </row>
@@ -547,7 +550,9 @@
           <t>- Crear, editar o eliminar cocteles
 - Crear modificadores
 - Crear o cancelar comandas
-- Cambiar el licor de un coctel de una comanda</t>
+- Cambiar el licor de un coctel de una comanda
+- Administrar los platos de la cocina
+- Consultar las reservas</t>
         </is>
       </c>
     </row>
@@ -568,14 +573,18 @@
 - Crear comandas para una mesa
 - Cambiar el licor de un coctel una vez, antes de la preparacion
 - Cancelar comandas en estado RECIBIDO
-- Consultar comandas</t>
+- Consultar comandas
+- Consultar sus propias comandas
+- Consultar la agenda de reservas y marcarlas como cumplidas o canceladas</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
           <t>- Crear, editar o eliminar cocteles y modificadores
 - Marcar productos como agotados
-- Avanzar el estado de una comanda en el tablero del bartender</t>
+- Avanzar el estado de una comanda en el tablero del bartender
+- Administrar los platos de la cocina
+- Calificar productos</t>
         </is>
       </c>
     </row>
@@ -596,7 +605,10 @@
 - Ver el detalle y los modificadores disponibles de un coctel
 - Enviar una comanda desde su mesa
 - Cambiar el licor de su coctel una vez, antes de la preparacion
-- Consultar el estado de su comanda</t>
+- Consultar el estado de su comanda
+- Consultar todas sus comandas
+- Calificar una vez cada coctel o plato
+- Reservar una mesa y consultar o cancelar sus reservas</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -605,7 +617,9 @@
 - Marcar productos como agotados
 - Ver las comandas de otras mesas o el tablero del bartender
 - Cambiar el estado de una comanda
-- Cancelar una comanda</t>
+- Cancelar una comanda
+- Ver las reservas de otras personas
+- Calificar dos veces el mismo producto</t>
         </is>
       </c>
     </row>
@@ -620,7 +634,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F24"/>
+  <dimension ref="A1:F36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -1399,6 +1413,390 @@
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Ver receta de referencia (TheCocktailDB)</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>GET /api/v1/menu/{id}/receta</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Ver los platos de la cocina</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>GET /api/v1/platos</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F26" s="4" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Crear, editar o eliminar platos</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>POST, PUT, DELETE /api/v1/platos</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Marcar plato agotado o disponible</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>PATCH /api/v1/platos/{id}/disponibilidad</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Consultar mis comandas</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>GET /api/v1/pedidos/mias</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Ver calificaciones y opiniones</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>GET /api/v1/resenas y /resenas/resumen</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Calificar un coctel o plato</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>POST /api/v1/resenas</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Reservar una mesa</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>POST /api/v1/reservas</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>Consultar la agenda de reservas</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>GET /api/v1/reservas</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>Consultar mis reservas</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>GET /api/v1/reservas/mias</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F34" s="4" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Marcar reserva cumplida o cancelada</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>PATCH /api/v1/reservas/{id}/estado</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F35" s="4" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>Cancelar una reserva</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>DELETE /api/v1/reservas/{id}</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F36" s="4" t="inlineStr">
+        <is>
+          <t>SI (solo la suya)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>